<commit_message>
adding columns to masterfile
</commit_message>
<xml_diff>
--- a/tests/data/example_masterfile.xlsx
+++ b/tests/data/example_masterfile.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stef/UCL/rred-reports/tests/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katiebuntic/projects/rred-reports/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB2BC22-D4D4-A94F-B74F-47D8BFF99187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78C3BA93-52A2-9049-A7EF-4770735AFDFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{1F5F4F09-FFBF-FF42-8606-4D2782A9E922}"/>
+    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{1F5F4F09-FFBF-FF42-8606-4D2782A9E922}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2311" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="219">
   <si>
     <t>reg_rr_title</t>
   </si>
@@ -687,6 +687,15 @@
   </si>
   <si>
     <t>11_2021-22-test</t>
+  </si>
+  <si>
+    <t>reg_deis_status</t>
+  </si>
+  <si>
+    <t>reg_lan</t>
+  </si>
+  <si>
+    <t>reg_lan_tum</t>
   </si>
 </sst>
 </file>
@@ -740,11 +749,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1059,7 +1070,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01BC0FAF-0515-DD4A-8720-9B9E6959245E}">
-  <dimension ref="A1:BR41"/>
+  <dimension ref="A1:BV41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1068,10 +1079,10 @@
     <col min="31" max="33" width="11" style="2"/>
     <col min="62" max="62" width="26.5" style="2" customWidth="1"/>
     <col min="66" max="66" width="38" customWidth="1"/>
-    <col min="70" max="70" width="22" customWidth="1"/>
+    <col min="74" max="74" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>176</v>
       </c>
@@ -1276,14 +1287,23 @@
       <c r="BP1" t="s">
         <v>65</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="BT1" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="BU1" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="BV1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="2" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>67</v>
       </c>
@@ -1488,11 +1508,13 @@
       <c r="BP2" t="s">
         <v>69</v>
       </c>
-      <c r="BQ2" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS2" s="4"/>
+      <c r="BT2" s="4"/>
     </row>
-    <row r="3" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -1697,11 +1719,13 @@
       <c r="BP3" t="s">
         <v>69</v>
       </c>
-      <c r="BQ3" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS3" s="4"/>
+      <c r="BT3" s="4"/>
     </row>
-    <row r="4" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>210</v>
       </c>
@@ -1906,11 +1930,13 @@
       <c r="BP4" t="s">
         <v>122</v>
       </c>
-      <c r="BQ4" s="1" t="s">
+      <c r="BR4" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="BS4" s="4"/>
+      <c r="BT4" s="4"/>
     </row>
-    <row r="5" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>211</v>
       </c>
@@ -2115,11 +2141,13 @@
       <c r="BP5" t="s">
         <v>69</v>
       </c>
-      <c r="BQ5" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS5" s="4"/>
+      <c r="BT5" s="4"/>
     </row>
-    <row r="6" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>212</v>
       </c>
@@ -2324,11 +2352,13 @@
       <c r="BP6" t="s">
         <v>69</v>
       </c>
-      <c r="BQ6" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS6" s="4"/>
+      <c r="BT6" s="4"/>
     </row>
-    <row r="7" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>213</v>
       </c>
@@ -2533,11 +2563,13 @@
       <c r="BP7" t="s">
         <v>69</v>
       </c>
-      <c r="BQ7" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS7" s="4"/>
+      <c r="BT7" s="4"/>
     </row>
-    <row r="8" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>214</v>
       </c>
@@ -2742,14 +2774,16 @@
       <c r="BP8" t="s">
         <v>69</v>
       </c>
-      <c r="BQ8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BR8" t="s">
+      <c r="BR8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS8" s="4"/>
+      <c r="BT8" s="4"/>
+      <c r="BV8" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>215</v>
       </c>
@@ -2954,11 +2988,13 @@
       <c r="BP9" t="s">
         <v>69</v>
       </c>
-      <c r="BQ9" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS9" s="4"/>
+      <c r="BT9" s="4"/>
     </row>
-    <row r="10" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>67</v>
       </c>
@@ -3163,11 +3199,13 @@
       <c r="BP10" t="s">
         <v>69</v>
       </c>
-      <c r="BQ10" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS10" s="4"/>
+      <c r="BT10" s="4"/>
     </row>
-    <row r="11" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>67</v>
       </c>
@@ -3372,11 +3410,13 @@
       <c r="BP11" t="s">
         <v>69</v>
       </c>
-      <c r="BQ11" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS11" s="4"/>
+      <c r="BT11" s="4"/>
     </row>
-    <row r="12" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>78</v>
       </c>
@@ -3581,11 +3621,13 @@
       <c r="BP12" t="s">
         <v>69</v>
       </c>
-      <c r="BQ12" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR12" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS12" s="4"/>
+      <c r="BT12" s="4"/>
     </row>
-    <row r="13" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>105</v>
       </c>
@@ -3790,11 +3832,13 @@
       <c r="BP13" t="s">
         <v>69</v>
       </c>
-      <c r="BQ13" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR13" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS13" s="4"/>
+      <c r="BT13" s="4"/>
     </row>
-    <row r="14" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>111</v>
       </c>
@@ -3999,11 +4043,13 @@
       <c r="BP14" t="s">
         <v>69</v>
       </c>
-      <c r="BQ14" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR14" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS14" s="4"/>
+      <c r="BT14" s="4"/>
     </row>
-    <row r="15" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>67</v>
       </c>
@@ -4208,11 +4254,13 @@
       <c r="BP15" t="s">
         <v>69</v>
       </c>
-      <c r="BQ15" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS15" s="4"/>
+      <c r="BT15" s="4"/>
     </row>
-    <row r="16" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>78</v>
       </c>
@@ -4417,11 +4465,13 @@
       <c r="BP16" t="s">
         <v>69</v>
       </c>
-      <c r="BQ16" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR16" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS16" s="4"/>
+      <c r="BT16" s="4"/>
     </row>
-    <row r="17" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>105</v>
       </c>
@@ -4626,11 +4676,13 @@
       <c r="BP17" t="s">
         <v>69</v>
       </c>
-      <c r="BQ17" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS17" s="4"/>
+      <c r="BT17" s="4"/>
     </row>
-    <row r="18" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>111</v>
       </c>
@@ -4835,11 +4887,13 @@
       <c r="BP18" t="s">
         <v>69</v>
       </c>
-      <c r="BQ18" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR18" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS18" s="4"/>
+      <c r="BT18" s="4"/>
     </row>
-    <row r="19" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>67</v>
       </c>
@@ -5044,11 +5098,13 @@
       <c r="BP19" t="s">
         <v>69</v>
       </c>
-      <c r="BQ19" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR19" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS19" s="4"/>
+      <c r="BT19" s="4"/>
     </row>
-    <row r="20" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>78</v>
       </c>
@@ -5253,11 +5309,13 @@
       <c r="BP20" t="s">
         <v>69</v>
       </c>
-      <c r="BQ20" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR20" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS20" s="4"/>
+      <c r="BT20" s="4"/>
     </row>
-    <row r="21" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>105</v>
       </c>
@@ -5462,11 +5520,13 @@
       <c r="BP21" t="s">
         <v>69</v>
       </c>
-      <c r="BQ21" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS21" s="4"/>
+      <c r="BT21" s="4"/>
     </row>
-    <row r="22" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>111</v>
       </c>
@@ -5671,14 +5731,16 @@
       <c r="BP22" t="s">
         <v>69</v>
       </c>
-      <c r="BQ22" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BR22" t="s">
+      <c r="BR22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS22" s="4"/>
+      <c r="BT22" s="4"/>
+      <c r="BV22" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="23" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -5883,11 +5945,13 @@
       <c r="BP23" t="s">
         <v>69</v>
       </c>
-      <c r="BQ23" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR23" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS23" s="4"/>
+      <c r="BT23" s="4"/>
     </row>
-    <row r="24" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -6092,11 +6156,13 @@
       <c r="BP24" t="s">
         <v>69</v>
       </c>
-      <c r="BQ24" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR24" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS24" s="4"/>
+      <c r="BT24" s="4"/>
     </row>
-    <row r="25" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>105</v>
       </c>
@@ -6301,11 +6367,13 @@
       <c r="BP25" t="s">
         <v>69</v>
       </c>
-      <c r="BQ25" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR25" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS25" s="4"/>
+      <c r="BT25" s="4"/>
     </row>
-    <row r="26" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -6510,11 +6578,13 @@
       <c r="BP26" t="s">
         <v>69</v>
       </c>
-      <c r="BQ26" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR26" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS26" s="4"/>
+      <c r="BT26" s="4"/>
     </row>
-    <row r="27" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -6719,11 +6789,13 @@
       <c r="BP27" t="s">
         <v>69</v>
       </c>
-      <c r="BQ27" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR27" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS27" s="4"/>
+      <c r="BT27" s="4"/>
     </row>
-    <row r="28" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>67</v>
       </c>
@@ -6928,11 +7000,13 @@
       <c r="BP28" t="s">
         <v>69</v>
       </c>
-      <c r="BQ28" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR28" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS28" s="4"/>
+      <c r="BT28" s="4"/>
     </row>
-    <row r="29" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>78</v>
       </c>
@@ -7137,11 +7211,13 @@
       <c r="BP29" t="s">
         <v>69</v>
       </c>
-      <c r="BQ29" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR29" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS29" s="4"/>
+      <c r="BT29" s="4"/>
     </row>
-    <row r="30" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>105</v>
       </c>
@@ -7346,11 +7422,13 @@
       <c r="BP30" t="s">
         <v>69</v>
       </c>
-      <c r="BQ30" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR30" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS30" s="4"/>
+      <c r="BT30" s="4"/>
     </row>
-    <row r="31" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>111</v>
       </c>
@@ -7555,11 +7633,13 @@
       <c r="BP31" t="s">
         <v>69</v>
       </c>
-      <c r="BQ31" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR31" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS31" s="4"/>
+      <c r="BT31" s="4"/>
     </row>
-    <row r="32" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -7764,11 +7844,13 @@
       <c r="BP32" t="s">
         <v>69</v>
       </c>
-      <c r="BQ32" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS32" s="4"/>
+      <c r="BT32" s="4"/>
     </row>
-    <row r="33" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>78</v>
       </c>
@@ -7973,11 +8055,13 @@
       <c r="BP33" t="s">
         <v>69</v>
       </c>
-      <c r="BQ33" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR33" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS33" s="4"/>
+      <c r="BT33" s="4"/>
     </row>
-    <row r="34" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>105</v>
       </c>
@@ -8182,11 +8266,13 @@
       <c r="BP34" t="s">
         <v>69</v>
       </c>
-      <c r="BQ34" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR34" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS34" s="4"/>
+      <c r="BT34" s="4"/>
     </row>
-    <row r="35" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>111</v>
       </c>
@@ -8391,14 +8477,16 @@
       <c r="BP35" t="s">
         <v>69</v>
       </c>
-      <c r="BQ35" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BR35" t="s">
+      <c r="BR35" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS35" s="4"/>
+      <c r="BT35" s="4"/>
+      <c r="BV35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>174</v>
       </c>
@@ -8603,14 +8691,16 @@
       <c r="BP36" t="s">
         <v>69</v>
       </c>
-      <c r="BQ36" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BR36" t="s">
+      <c r="BR36" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS36" s="4"/>
+      <c r="BT36" s="4"/>
+      <c r="BV36" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="37" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>67</v>
       </c>
@@ -8815,11 +8905,13 @@
       <c r="BP37" t="s">
         <v>69</v>
       </c>
-      <c r="BQ37" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR37" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS37" s="4"/>
+      <c r="BT37" s="4"/>
     </row>
-    <row r="38" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>78</v>
       </c>
@@ -9024,11 +9116,13 @@
       <c r="BP38" t="s">
         <v>69</v>
       </c>
-      <c r="BQ38" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR38" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS38" s="4"/>
+      <c r="BT38" s="4"/>
     </row>
-    <row r="39" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>105</v>
       </c>
@@ -9233,11 +9327,13 @@
       <c r="BP39" t="s">
         <v>69</v>
       </c>
-      <c r="BQ39" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="BR39" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS39" s="4"/>
+      <c r="BT39" s="4"/>
     </row>
-    <row r="40" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>111</v>
       </c>
@@ -9442,14 +9538,16 @@
       <c r="BP40" t="s">
         <v>69</v>
       </c>
-      <c r="BQ40" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BR40" t="s">
+      <c r="BR40" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS40" s="4"/>
+      <c r="BT40" s="4"/>
+      <c r="BV40" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="41" spans="1:70" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:74" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>174</v>
       </c>
@@ -9654,10 +9752,12 @@
       <c r="BP41" t="s">
         <v>69</v>
       </c>
-      <c r="BQ41" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BR41" t="s">
+      <c r="BR41" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS41" s="4"/>
+      <c r="BT41" s="4"/>
+      <c r="BV41" t="s">
         <v>157</v>
       </c>
     </row>

</xml_diff>